<commit_message>
Make long sample changed-only (no unchanged rows, ~2 pages)
</commit_message>
<xml_diff>
--- a/examples/japanese-long-comparison.xlsx
+++ b/examples/japanese-long-comparison.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
   <si>
     <t>新旧対照表</t>
   </si>
@@ -37,30 +37,12 @@
     <t>第1条 目的</t>
   </si>
   <si>
-    <t>本条（目的）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-  </si>
-  <si>
-    <t>変更なし</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>第2条 定義</t>
-  </si>
-  <si>
-    <t>本条（定義）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-  </si>
-  <si>
-    <t>第3条 適用範囲</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans JP"/>
-      </rPr>
-      <t>本条（適用範囲）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>本条（目的）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
     </r>
     <r>
       <rPr>
@@ -73,28 +55,13 @@
     </r>
   </si>
   <si>
-    <t>本条（適用範囲）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
+    <t>本条（目的）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
   </si>
   <si>
     <t>変更</t>
   </si>
   <si>
-    <t>第4条 服務規律</t>
-  </si>
-  <si>
-    <t>本条（服務規律）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-  </si>
-  <si>
-    <t>第5条 勤務時間</t>
-  </si>
-  <si>
-    <t>本条（勤務時間）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-  </si>
-  <si>
-    <t>第6条 休憩</t>
-  </si>
-  <si>
-    <t>本条（休憩）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
+    <t/>
   </si>
   <si>
     <t>第7条 休日</t>
@@ -121,33 +88,15 @@
     <t>本条（休日）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
   </si>
   <si>
-    <t>第8条 休暇</t>
-  </si>
-  <si>
-    <t>本条（休暇）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-  </si>
-  <si>
-    <t>第9条 給与</t>
-  </si>
-  <si>
-    <t>本条（給与）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-  </si>
-  <si>
-    <t>第11条 退職金</t>
-  </si>
-  <si>
-    <t>本条（退職金）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-  </si>
-  <si>
-    <t>第12条 出張旅費</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans JP"/>
-      </rPr>
-      <t>本条（出張旅費）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
+    <t>第13条 在宅勤務</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>本条（在宅勤務）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
     </r>
     <r>
       <rPr>
@@ -160,48 +109,18 @@
     </r>
   </si>
   <si>
-    <t>本条（出張旅費）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-  </si>
-  <si>
-    <t>第13条 在宅勤務</t>
-  </si>
-  <si>
     <t>本条（在宅勤務）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
   </si>
   <si>
-    <t>第14条 服装規定</t>
-  </si>
-  <si>
-    <t>本条（服装規定）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-  </si>
-  <si>
-    <t>第15条 情報管理</t>
-  </si>
-  <si>
-    <t>本条（情報管理）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-  </si>
-  <si>
-    <t>第16条 安全衛生</t>
-  </si>
-  <si>
-    <t>本条（安全衛生）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-  </si>
-  <si>
-    <t>第17条 懲戒</t>
-  </si>
-  <si>
-    <t>本条（懲戒）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-  </si>
-  <si>
-    <t>第18条 教育研修</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans JP"/>
-      </rPr>
-      <t>本条（教育研修）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
+    <t>第19条 福利厚生</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>本条（福利厚生）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
     </r>
     <r>
       <rPr>
@@ -214,19 +133,7 @@
     </r>
   </si>
   <si>
-    <t>本条（教育研修）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-  </si>
-  <si>
-    <t>第19条 福利厚生</t>
-  </si>
-  <si>
     <t>本条（福利厚生）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-  </si>
-  <si>
-    <t>第20条 雑則</t>
-  </si>
-  <si>
-    <t>本条（雑則）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
   </si>
   <si>
     <t>第21条 附則</t>
@@ -333,11 +240,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -681,7 +588,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -715,361 +622,106 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" ht="116" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" ht="164" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="4" t="s">
         <v>8</v>
       </c>
+      <c r="D3" s="5" t="s">
+        <v>9</v>
+      </c>
       <c r="E3" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" ht="164" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" ht="116" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="5" ht="164" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>15</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" ht="164" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>9</v>
       </c>
+      <c r="E6" s="3" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="6" ht="116" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" ht="116" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" ht="52" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" ht="116" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>8</v>
+        <v>24</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" ht="164" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" ht="116" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" ht="116" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" ht="116" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" ht="164" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" ht="116" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="15" ht="116" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="16" ht="116" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="17" ht="116" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="18" ht="116" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19" ht="164" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" ht="116" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="21" ht="116" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="22" ht="52" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="23" ht="116" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Diversify long sample: varied revision types across 2 pages
</commit_message>
<xml_diff>
--- a/examples/japanese-long-comparison.xlsx
+++ b/examples/japanese-long-comparison.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="45">
   <si>
     <t>新旧対照表</t>
   </si>
@@ -42,20 +42,27 @@
         <sz val="10"/>
         <rFont val="Noto Sans JP"/>
       </rPr>
-      <t>本条（目的）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <color rgb="FFFF0000"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans JP"/>
-      </rPr>
-      <t>また、本改定により、適用対象および手続の一部を変更し、契約社員を含む全従業員に適用することとした。</t>
-    </r>
-  </si>
-  <si>
-    <t>本条（目的）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
+      <t>本規則は、株式会社サンプルの従業員</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <color rgb="FFFF0000"/>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>（契約社員を含む。）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>の労働条件および服務規律を定めることを目的とする。</t>
+    </r>
+  </si>
+  <si>
+    <t>本規則は、株式会社サンプルの従業員の労働条件および服務規律を定めることを目的とする。</t>
   </si>
   <si>
     <t>変更</t>
@@ -64,102 +71,350 @@
     <t/>
   </si>
   <si>
-    <t>第7条 休日</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans JP"/>
-      </rPr>
-      <t>本条（休日）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <color rgb="FFFF0000"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans JP"/>
-      </rPr>
-      <t>また、本改定により、適用対象および手続の一部を変更し、契約社員を含む全従業員に適用することとした。</t>
-    </r>
-  </si>
-  <si>
-    <t>本条（休日）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-  </si>
-  <si>
-    <t>第13条 在宅勤務</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans JP"/>
-      </rPr>
-      <t>本条（在宅勤務）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <color rgb="FFFF0000"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans JP"/>
-      </rPr>
-      <t>また、本改定により、適用対象および手続の一部を変更し、契約社員を含む全従業員に適用することとした。</t>
-    </r>
-  </si>
-  <si>
-    <t>本条（在宅勤務）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-  </si>
-  <si>
-    <t>第19条 福利厚生</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans JP"/>
-      </rPr>
-      <t>本条（福利厚生）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <color rgb="FFFF0000"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans JP"/>
-      </rPr>
-      <t>また、本改定により、適用対象および手続の一部を変更し、契約社員を含む全従業員に適用することとした。</t>
-    </r>
-  </si>
-  <si>
-    <t>本条（福利厚生）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
-  </si>
-  <si>
-    <t>第21条 附則</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u/>
-        <color rgb="FFFF0000"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans JP"/>
-      </rPr>
-      <t>本規程は、本改定後、所定の手続を経て施行する。改定後の規定は、施行日以後に発生した事象について適用するものとする。</t>
+    <t>第3条 適用範囲</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>本規則は、会社に在籍するすべての正社員</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <color rgb="FFFF0000"/>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>および契約社員</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>に適用する。</t>
+    </r>
+  </si>
+  <si>
+    <t>本規則は、会社に在籍するすべての正社員に適用する。</t>
+  </si>
+  <si>
+    <t>第4条 勤務時間</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>始業時刻は午前9時、終業時刻は午後6時とし、休憩時間は60分とする。</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <color rgb="FFFF0000"/>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>なお、コアタイムを午前10時から午後3時までとするフレックスタイム制を導入する。</t>
+    </r>
+  </si>
+  <si>
+    <t>始業時刻は午前9時、終業時刻は午後6時とし、休憩時間は60分とする。</t>
+  </si>
+  <si>
+    <t>第5条 賃金</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>賃金は、毎月</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <color rgb="FFFF0000"/>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>日に締め切り、</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <color rgb="FFFF0000"/>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>当</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>月25日に支払う。</t>
+    </r>
+  </si>
+  <si>
+    <t>賃金は、毎月末日に締め切り、翌月25日に支払う。</t>
+  </si>
+  <si>
+    <t>第6条 時間外労働</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>会社は、業務の都合により、従業員に時間外労働を命じることがある。</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <color rgb="FFFF0000"/>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>この場合において、時間外労働は月45時間、年360時間を上限とする。</t>
+    </r>
+  </si>
+  <si>
+    <t>会社は、業務の都合により、従業員に時間外労働を命じることがある。</t>
+  </si>
+  <si>
+    <t>第8条 年次有給休暇</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>会社は、6か月間継続勤務し、所定労働日の8割以上出勤した従業員に対し、10日の年次有給休暇を付与する。</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <color rgb="FFFF0000"/>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>当該年次有給休暇は、半日単位および時間単位で取得することができる。</t>
+    </r>
+  </si>
+  <si>
+    <t>会社は、6か月間継続勤務し、所定労働日の8割以上出勤した従業員に対し、10日の年次有給休暇を付与する。</t>
+  </si>
+  <si>
+    <t>第9条 退職</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>従業員が自己の都合により退職しようとするときは、退職日の</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <color rgb="FFFF0000"/>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>日前までに届け出なければならない。</t>
+    </r>
+  </si>
+  <si>
+    <t>従業員が自己の都合により退職しようとするときは、退職日の14日前までに届け出なければならない。</t>
+  </si>
+  <si>
+    <t>第10条 育児休業</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <color rgb="FFFF0000"/>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>従業員は、1歳に満たない子を養</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>育</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <color rgb="FFFF0000"/>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>するため、育</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>児休業</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <color rgb="FFFF0000"/>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>を取得</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>する</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <color rgb="FFFF0000"/>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>ことができる。対象者、期間その他必要な</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>事項は、育児・介護休業規程に</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <color rgb="FFFF0000"/>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>定めるところに</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>よる。</t>
+    </r>
+  </si>
+  <si>
+    <t>育児休業に関する事項は、別に定める育児・介護休業規程による。</t>
+  </si>
+  <si>
+    <t>第12条 ハラスメントの防止</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <color rgb="FFFF0000"/>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>会社は、職場におけるあらゆるハラスメントを防止するため、必要な措置を講じる。従業員は、相互に人格を尊重し、ハラスメントに該当する行為を行ってはならない。</t>
     </r>
   </si>
   <si>
     <t>追加</t>
   </si>
   <si>
-    <t>第10条 賞与</t>
-  </si>
-  <si>
-    <t>本条（賞与）に関する事項は、本規程の定めるところによる。会社および従業員は、相互の信頼に基づき、本条の趣旨を理解のうえ、誠実にこれを遵守しなければならない。具体的な取扱いおよび手続については、別途定める運用基準または細則によるものとし、必要に応じて適宜見直すことができるものとする。</t>
+    <t>第14条 安全衛生</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <color rgb="FFFF0000"/>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>会社は、従業員の安全および健康を確保するため、必要な措置を講じる。従業員は、会社が行う安全衛生に関する措置に協力しなければならない。</t>
+    </r>
+  </si>
+  <si>
+    <t>第18条 懲戒</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>従業員が次の各号</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <color rgb="FFFF0000"/>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>のいずれか</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans JP"/>
+      </rPr>
+      <t>に該当する場合は、懲戒処分を行うものとする。</t>
+    </r>
+  </si>
+  <si>
+    <t>従業員が次の各号に該当する場合は、懲戒処分を行うものとする。</t>
+  </si>
+  <si>
+    <t>第15条 社宅</t>
+  </si>
+  <si>
+    <t>会社は、従業員の福利厚生のため社宅を貸与することがある。</t>
   </si>
   <si>
     <t>削除</t>
+  </si>
+  <si>
+    <t>第20条 出向</t>
+  </si>
+  <si>
+    <t>会社は、業務上の必要により、従業員に出向を命じることがある。</t>
   </si>
 </sst>
 </file>
@@ -588,7 +843,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -622,7 +877,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" ht="164" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" ht="52" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
@@ -639,7 +894,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" ht="164" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
@@ -656,7 +911,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" ht="164" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" ht="68" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
@@ -673,7 +928,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" ht="164" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>17</v>
       </c>
@@ -690,7 +945,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" ht="52" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" ht="68" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>20</v>
       </c>
@@ -698,29 +953,148 @@
         <v>21</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" ht="116" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" ht="68" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>10</v>
+      <c r="B8" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="E8" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" ht="52" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" ht="68" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" ht="68" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" ht="68" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>